<commit_message>
akademik: Gorev-8 tam-metin teyidi islendi (4 hucre degisti) + xlsx senkron + kol2/33 log
- #2 C1 c->a (yineleme yok, yalniz DBR dongusu+atif)
- #1/#4/#34 C6 cift-kutup->yalniz-risk (pozitif=PD->C5 veya risk-yanli rol)
- #7/#30 C1c, #8 cift-kutup tam-metinle dogrulandi (alinti+sayfa)
- xlsx guncel md'den yeniden uretildi; kodlama KILITLENDI

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AfwpDUUVNN675U8HGdboQJ
</commit_message>
<xml_diff>
--- a/projects/yz-yabancidil-derleme/kol2/27-kodlama-tablosu.xlsx
+++ b/projects/yz-yabancidil-derleme/kol2/27-kodlama-tablosu.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C8_kodlama" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C1-C8 Kodlama (v1.2+G8)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +28,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="3">
@@ -58,10 +62,10 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -431,21 +435,21 @@
   <dimension ref="A1:O26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="46" customWidth="1" min="15" max="15"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="48" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -558,7 +562,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1c (v1.2)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -568,12 +572,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>4 (tasarımcı) · güçlenme</t>
+          <t>4 (tasarımcı)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>accuracy/error tartışılıyor; validate</t>
+          <t>accuracy/error; validate</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -583,7 +587,7 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>etik, emek</t>
+          <t>RİSK: etik, emek (Görev-8: pozitif PD→C5, çift-kutup kaldırıldı)</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -598,7 +602,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>'develop reading materials' — öğretmen GenAI ile okuma materyali üretir</t>
+          <t>'develop reading materials' + 'iteratively'</t>
         </is>
       </c>
     </row>
@@ -635,7 +639,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1a (Görev-8)</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -660,12 +664,12 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>bias, etik, veri-mahremiyet, eşitlik</t>
+          <t>RİSK: bias, etik, mahremiyet, eşitlik + POZİTİF: güçlenme/faillik (v1.2)</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>genel; L2; karma (design-based, quasi-exp+görüşme)</t>
+          <t>genel; L2; karma</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -675,7 +679,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>AI-generated materials etkililiği test ediliyor</t>
+          <t>AI-gen materials etkililiği; yineleme yok—yalnız DBR döngüsü ('two iterative cycles', s.2) + atıf ('revise prompts iteratively' Ahn 2024, s.5) → C1a (Görev-8)</t>
         </is>
       </c>
     </row>
@@ -712,7 +716,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1c (v1.2)</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -737,12 +741,12 @@
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>etik, emek</t>
+          <t>RİSK: etik, emek</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>akademik yazma; L2; nitel (case)</t>
+          <t>akademik yazma; L2; nitel</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -752,7 +756,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>ESAP materials development with GenAI</t>
+          <t>ESAP materials development + iterative</t>
         </is>
       </c>
     </row>
@@ -799,12 +803,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2 (v1.2)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>HALÜSİNASYON + uzman-denetim + accuracy (güçlü C4)</t>
+          <t>HALÜSİNASYON+uzman-denetim (güçlü)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -814,7 +818,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>etik, emek, bias, dijital-uçurum, eşitlik (zengin)</t>
+          <t>RİSK: etik, emek, bias, dijital-uçurum, eşitlik (zengin) (Görev-8: pozitif yok, çift-kutup kaldırıldı)</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -829,7 +833,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>AI-generated instructional videos; expert review + hallucination</t>
+          <t>'We developed' AIIV; rol='reshaping...additional demands' risk-yanlı+atıf (s.19) → yalnız-risk (Görev-8)</t>
         </is>
       </c>
     </row>
@@ -866,7 +870,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1c (v1.2)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -891,12 +895,12 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>bias</t>
+          <t>RİSK: bias</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>okuma, söz varlığı; L2; karma (quasi-exp+içerik)</t>
+          <t>okuma/söz varlığı; L2; karma</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -906,7 +910,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>generating Arabic personalized materials</t>
+          <t>generating Arabic materials + iterative</t>
         </is>
       </c>
     </row>
@@ -943,7 +947,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1c (uzlaşı)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -953,7 +957,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>5 (geliştirici) · PROFESYONEL KİMLİK (güçlü)</t>
+          <t>4 (v1.2)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -968,12 +972,12 @@
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>bias, eşitlik, etik, emek</t>
+          <t>RİSK: bias, eşitlik, etik, emek + POZİTİF: öğretmen rol dönüşümü (üç-aşamalı TPI) (uzlaşı)</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>okuma; L2; nitel (case, 2 öğretmen)</t>
+          <t>okuma; L2; nitel (2 öğretmen)</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -983,7 +987,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>teacher professional identity + teacher-generated reading materials</t>
+          <t>'refine/adjust prompts iteratively'; TPI dönüşümü</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1014,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Öğretim etkinliği/materyali (korpus+GenAI)</t>
+          <t>Öğretim etkinliği/materyali</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1020,7 +1024,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>C1a/C1c</t>
+          <t>C1c (v1.2)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1030,7 +1034,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>4 · ÖĞRETMEN FAİLLİĞİ (açık)</t>
+          <t>4 · öğretmen failliği</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -1045,7 +1049,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>bias, etik</t>
+          <t>RİSK: bias, etik + POZİTİF: öğretmen failliği (v1.2)</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -1060,7 +1064,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>'Activity generated by ChatGPT' (Student 7); teacher agency</t>
+          <t>'Activity generated by ChatGPT'; teacher agency; 'students refined it in subsequent iterations' (s.7) → C1c teyit (Görev-8)</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1091,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Öyküye-dayalı okuma materyali (otomatik pipeline)</t>
+          <t>Öyküye-dayalı okuma materyali (pipeline)</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1097,7 +1101,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>C1a (pipeline≈C1d)</t>
+          <t>C1e (v1.2)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1112,7 +1116,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>HALÜSİNASYON + uzman-değerlendirme + VALİDASYON (güçlü)</t>
+          <t>HALÜSİNASYON+uzman-değerlendirme+VALİDASYON (güçlü)</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1122,12 +1126,12 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>etik, bias, eşitlik</t>
+          <t>RİSK: etik, bias, eşitlik + POZİTİF: güçlenme/faillik (v1.2)</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>okuma, söz varlığı; L2; karma (ön/son+validasyon)</t>
+          <t>okuma/söz varlığı; L2; karma</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1137,7 +1141,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>automated pipeline + expert evaluation/validation</t>
+          <t>automated pipeline; 'roles...shifting from simple content creators to content curators and editors' (s.15) → çift-kutup teyit (Görev-8)</t>
         </is>
       </c>
     </row>
@@ -1169,12 +1173,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>İngilizce-EFL (çok-kültürlü)</t>
+          <t>İngilizce-EFL</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>C1c</t>
+          <t>C1c′ (v1.2)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1184,7 +1188,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>3 (kolaylaştırıcı) · güçlenme</t>
+          <t>3 (kolaylaştırıcı)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1199,12 +1203,12 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>eşitlik, etik, emek</t>
+          <t>RİSK: eşitlik, etik, emek + POZİTİF: öğrenen güçlenme/faillik (v1.2)</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>yazma/söz varlığı/dilbilgisi; L2; nitel (11 öğr.)</t>
+          <t>yazma/söz varlığı/dilbilgisi; L2; nitel</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1214,7 +1218,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>students integrate GenAI into digital multimodal composition</t>
+          <t>students integrate GenAI into DMC</t>
         </is>
       </c>
     </row>
@@ -1276,12 +1280,12 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>eşitlik, etik, YAZARLIK, bias</t>
+          <t>RİSK: eşitlik, etik, YAZARLIK, bias</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>yazma/konuşma; L2; karma (case)</t>
+          <t>yazma/konuşma; L2; karma</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1291,7 +1295,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>teachers collaborate with AI chatbots to create materials</t>
+          <t>collaborate with AI chatbots (co-creation)</t>
         </is>
       </c>
     </row>
@@ -1353,12 +1357,12 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>etik, bias, emek, mahremiyet</t>
+          <t>RİSK: etik, bias, emek, mahremiyet + POZİTİF: güçlenme/faillik (v1.2)</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>genel; L2; Ar-Ge/ADDIE (prototip)</t>
+          <t>genel; L2; Ar-Ge/ADDIE</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1368,7 +1372,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>develop/produce/test instructional learning media (product)</t>
+          <t>develop/produce/test instructional media</t>
         </is>
       </c>
     </row>
@@ -1400,7 +1404,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>İngilizce (Global Englishes)</t>
+          <t>İngilizce (GE)</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1415,7 +1419,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>5 · ÖĞRETMEN FAİLLİĞİ (açık) · güçlenme</t>
+          <t>4 (v1.2)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1430,12 +1434,12 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>bias, etik, emek</t>
+          <t>RİSK: bias, etik, emek + POZİTİF: öğretmen failliği/güçlenme (v1.2)</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>okuma/dinleme; L2; nitel (IPA, 280 öğr./2 öğretmen)</t>
+          <t>okuma/dinleme; L2; nitel (IPA)</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1445,7 +1449,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>teachers select GenAI to generate GE reading/listening materials</t>
+          <t>teachers select GenAI to generate GE materials; teacher agency açık</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1486,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>C1c</t>
+          <t>C1c′ (v1.2)</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1507,12 +1511,12 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>YAZARLIK ETİĞİ + veri-mahremiyet + etik (zengin)</t>
+          <t>RİSK: YAZARLIK etiği, mahremiyet, etik + POZİTİF: yaratıcı işbirlikçi rol (uzlaşı)</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>konuşma/yazma(senaryo); L2; nitel (80 öğr.)</t>
+          <t>konuşma/yazma(senaryo); L2; nitel</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1522,7 +1526,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>students produce EFL podcasts (script→ideas→editing) with GenAI</t>
+          <t>students produce EFL podcasts (script→ideas→editing)</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1578,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>CEFR + HALÜSİNASYON + accuracy/inaccurate (güçlü)</t>
+          <t>CEFR+HALÜSİNASYON+accuracy (güçlü)</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1584,12 +1588,12 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>bias, etik, mahremiyet</t>
+          <t>RİSK: bias, etik, mahremiyet</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>okuma/söz varlığı; L2; nicel (ön/son)</t>
+          <t>okuma/söz varlığı; L2; nicel</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1631,12 +1635,12 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>İngilizce-EFL (öğretmen-eğitimi)</t>
+          <t>İngilizce-EFL</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1c (v1.2)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1656,17 +1660,17 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>AI/dijital okuryazarlık, prompt müh., öğretmen eğitimi (zengin)</t>
+          <t>AI/dijital okuryazarlık, prompt müh., öğretmen eğitimi</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>etik, emek</t>
+          <t>RİSK: etik, emek + POZİTİF: güçlenme/faillik (v1.2)</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>genel; L2; karma (action research+anket 270)</t>
+          <t>genel; L2; karma (action research)</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1676,7 +1680,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>creating personalised storybooks + lesson plans (PPT demo)</t>
+          <t>creating storybooks + lesson plans + iterative</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1717,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1c (v1.2)</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1728,7 +1732,7 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>CEFR + HALÜSİNASYON + accuracy/alignment/validated (güçlü)</t>
+          <t>CEFR+HALÜSİNASYON+accuracy/validated</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1738,7 +1742,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>emek, mahremiyet</t>
+          <t>RİSK: emek, mahremiyet</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -1753,7 +1757,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>ChatGPT designs teaching materials for Romanian-FL</t>
+          <t>'we developed' RFL materials + iterative</t>
         </is>
       </c>
     </row>
@@ -1775,7 +1779,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Sistem/Öğretmen</t>
+          <t>Sistem (araştırmacı-kurmalı)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1790,7 +1794,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>C1d</t>
+          <t>C1e (v1.2)</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1800,12 +1804,12 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>4 · iş-yükü</t>
+          <t>1 (uzlaşı)</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>CEFR + VERİFİKASYON + uzman-değerlendirme + alignment (çok güçlü)</t>
+          <t>CEFR+VERİFİKASYON+uzman-değerlendirme (çok güçlü)</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1815,12 +1819,12 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>etik, bias, emek</t>
+          <t>RİSK: etik, bias, emek</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>genel; L2; nicel (18 öğretmen/139 öğr. değerlendirme)</t>
+          <t>genel; L2; nicel</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1830,7 +1834,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>RAG+multi-agent framework for EFL content generation</t>
+          <t>'we designed and implemented the CCGF'; öğretmen yalnız KÖR-DEĞERLENDİRİCİ</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1871,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1c (v1.2)</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -1892,12 +1896,12 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>bias, eşitlik, etik, AŞIRI-BAĞIMLILIK (zengin)</t>
+          <t>RİSK: bias, eşitlik, etik, AŞIRI-BAĞIMLILIK (zengin) + POZİTİF: güçlenme/faillik (v1.2)</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>kültür; L2; karma (case, 61 öğretmen)</t>
+          <t>kültür; L2; karma (61 öğretmen)</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -1907,7 +1911,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>teachers create culturally inclusive materials + evaluate GenAI outputs</t>
+          <t>teachers create culturally inclusive materials + evaluate; 'modify the outputs' + 'significant prompting' (s.8,10) → C1c teyit (Görev-8)</t>
         </is>
       </c>
     </row>
@@ -1929,7 +1933,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Öğretmen</t>
+          <t>Öğretmen (in-service, HE)</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1944,7 +1948,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1a′ (v1.2)</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1954,7 +1958,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>4 · güçlenme/iş-yükü</t>
+          <t>3 (uzlaşı) · anket-beyan (gözlenmedi)</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1969,12 +1973,12 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>bias, etik, emek, mahremiyet</t>
+          <t>RİSK: bias, etik, emek, mahremiyet (Görev-8: pozitif yalnız PD-talebi→C5, çift-kutup kaldırıldı)</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>değerlendirme(okuma/yazma/söz/dilbilgisi); L2; karma (anket)</t>
+          <t>değerlendirme; L2; karma (anket)</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -1984,7 +1988,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>create effective ChatGPT-generated test tasks (assessment)</t>
+          <t>ChatGPT-gen görev + doğruluk süzme; algı anketi; pozitif yalnız 'need for PD' (s.10,12) → yalnız-risk (Görev-8)</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2010,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Eş-üretim</t>
+          <t>Eş-üretim (öğrenci–YZ)</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -2021,7 +2025,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>C1c</t>
+          <t>C1c′ (uzlaşı)</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2036,7 +2040,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>CEFR + rubric + validation + hallucinate</t>
+          <t>CEFR+rubric+validation+hallucinate</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2046,7 +2050,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>YAZARLIK + bias + etik</t>
+          <t>RİSK: YAZARLIK, bias, etik</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -2061,7 +2065,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>controlled experiment: Human-only/Human-LLM/LLM-only creative writing (GFL)</t>
+          <t>40 GFL undergrad öğrenci üretici; Human-LLM creative writing</t>
         </is>
       </c>
     </row>
@@ -2098,7 +2102,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>C1a</t>
+          <t>C1c (v1.2)</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2113,7 +2117,7 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>CEFR + error/accuracy/alignment (sözcüksel denetim; güçlü)</t>
+          <t>CEFR+sözcüksel denetim (güçlü)</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2123,7 +2127,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>emek</t>
+          <t>RİSK: emek</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -2138,7 +2142,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>GenAI generates customized texts for absolute beginners (controlled)</t>
+          <t>generates beginner texts w/ lexical control + iterative</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2179,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>C1c</t>
+          <t>C1c′ (v1.2)</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2200,22 +2204,22 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>YAZARLIK, emek</t>
+          <t>RİSK: YAZARLIK, emek</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>okuma; L2; müdahale (ön/son anket+görüşme)</t>
+          <t>okuma; L2; müdahale</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>empirik; orta-zayıf (küçük)</t>
+          <t>empirik; orta-zayıf</t>
         </is>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>students created storybooks with CopyAI/GPT-3 (Fig. 3)</t>
+          <t>participants created storybooks (Fig.3)</t>
         </is>
       </c>
     </row>
@@ -2252,7 +2256,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>C1c</t>
+          <t>C1c′ (v1.2)</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2267,7 +2271,7 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>alignment + rubric + uzman-denetim + accuracy</t>
+          <t>alignment+rubric+uzman-denetim</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2277,12 +2281,12 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>bias, emek, AŞIRI-BAĞIMLILIK</t>
+          <t>RİSK: bias, emek, AŞIRI-BAĞIMLILIK</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>söz varlığı; L2; karma (ön/son, 80 öğr.)</t>
+          <t>söz varlığı; L2; karma (80 öğr.)</t>
         </is>
       </c>
       <c r="N24" s="2" t="inlineStr">
@@ -2292,7 +2296,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>students make comic-book digital stories via AI text-to-image</t>
+          <t>students co-create comic-book digital stories</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2328,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>İngilizce-EFL (Türkiye, ilkokul 1.sınıf)</t>
+          <t>İngilizce-EFL (Türkiye, ilkokul)</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -2349,17 +2353,17 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>AI/dijital okuryazarlık, prompt müh., öğretmen eğitimi (zengin)</t>
+          <t>AI/dijital okuryazarlık, prompt müh., öğretmen eğitimi</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>eşitlik, etik, emek, mahremiyet</t>
+          <t>RİSK: eşitlik, etik, emek, mahremiyet</t>
         </is>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>söz varlığı; L2; deneysel (ön/son, 40 öğr.)</t>
+          <t>söz varlığı; L2; deneysel</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -2369,7 +2373,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>DALL-E generates vocabulary cards (vs traditional)</t>
+          <t>DALL-E generates vocabulary cards</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2425,7 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>CEFR + accuracy/alignment/error</t>
+          <t>CEFR+accuracy/alignment/error</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2431,12 +2435,12 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>YAZARLIK, etik, emek, AŞIRI-BAĞIMLILIK</t>
+          <t>RİSK: YAZARLIK, etik, emek, AŞIRI-BAĞIMLILIK</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>yazma(IELTS); L2; karma (quasi-exp+görüşme)</t>
+          <t>yazma(IELTS); L2; karma</t>
         </is>
       </c>
       <c r="N26" s="2" t="inlineStr">
@@ -2446,7 +2450,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>AI-generated sample writings + personalized feedback (teacher-mediated)</t>
+          <t>AI sample writings + feedback (teacher-mediated, iterative)</t>
         </is>
       </c>
     </row>

</xml_diff>